<commit_message>
Update Insurance module, AI service, and Social features
</commit_message>
<xml_diff>
--- a/Data/Insurance Provider.xlsx
+++ b/Data/Insurance Provider.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vfzzz/Downloads/PetWell/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{15AA930C-F617-424D-90C8-E8D125B91FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46124032-F05F-B34C-8531-3520BCDC978D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="600" windowWidth="19200" windowHeight="19340" xr2:uid="{C7394F8D-4CC2-CE4F-A891-5C82920EF005}"/>
+    <workbookView xWindow="15120" yWindow="660" windowWidth="15120" windowHeight="17520" xr2:uid="{C7394F8D-4CC2-CE4F-A891-5C82920EF005}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Insurance Info" sheetId="1" r:id="rId1"/>
+    <sheet name="Glossary" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -58,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
   <si>
     <t xml:space="preserve">Insurance Provider </t>
   </si>
@@ -85,13 +86,115 @@
   </si>
   <si>
     <t>Annual Coverage(HKD)</t>
+  </si>
+  <si>
+    <t>Surgery</t>
+  </si>
+  <si>
+    <t>Overnight</t>
+  </si>
+  <si>
+    <t>Hospitalization</t>
+  </si>
+  <si>
+    <t>X-Ray &amp; Ultrasound</t>
+  </si>
+  <si>
+    <t>Lab Test</t>
+  </si>
+  <si>
+    <t>Medication</t>
+  </si>
+  <si>
+    <t>Consultation</t>
+  </si>
+  <si>
+    <t>Specialist Consultation</t>
+  </si>
+  <si>
+    <t>MRI &amp; CT Coverage</t>
+  </si>
+  <si>
+    <t>Cancer Cash</t>
+  </si>
+  <si>
+    <t>Additional Advanced Critical Illness Cash Benefit(Require Check Eligibility), 
+Additional Critial Illness Cash Benefit (Check Eligibility)</t>
+  </si>
+  <si>
+    <t>Eligibility</t>
+  </si>
+  <si>
+    <t>For cats and dogs aged 1-9 who have not suffered from specified critical illnesses before. The cash benefit can only be claimed once during a pet's lifetime.
+For cats and dogs aged 1–9 who have not suffered from specified critical illnesses before. The cash benefit can only be claimed once during a pet's lifetime.</t>
+  </si>
+  <si>
+    <t>For cats aged 1–11 who have not previously suffered from FIP before enrolment. There’s no age limit on renewal. This coverage can only be claimed once during a pet's lifetime.</t>
+  </si>
+  <si>
+    <t>Feline Infectious Peritonitis (FIP) Additional Coverage (Cat Only)</t>
+  </si>
+  <si>
+    <t>精選計劃</t>
+  </si>
+  <si>
+    <t>全方位計劃</t>
+  </si>
+  <si>
+    <t>尊寵計劃</t>
+  </si>
+  <si>
+    <t>珍寵計劃</t>
+  </si>
+  <si>
+    <t>為1-9歲及未曾患上指定危疾的貓狗提供的現金保障。此保障終身只能索償一次。
+為1-9歲及未曾患上指定危疾的貓狗提供的現金保障。此保障終身只能索償一次。</t>
+  </si>
+  <si>
+    <t>為1歲至11歲及投保前未曾患上貓傳染性腹膜炎的貓提供的額外保額，不設續保年齡限制。此保障終身只能索償一次。</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Additional Advanced Critical Illness Cash Benefit: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5 Critical Illnesses Covered:
+Epileptic Seizure, Quadriplegia, Patellar Luxation (Dislocation), Heart Failure, Stroke
+涵蓋 5 項危疾：
+癲癇發作、四肢癱瘓、髕骨脫臼、心臟衰竭、中風
+Additional Critical Illness Cash Benefit
+3 Critical Illnesses Covered:
+Epileptic Seizure, Quadriplegia, Patellar Luxation (Dislocation)
+涵蓋 3 項危疾：
+癲癇發作、四肢癱瘓、髕骨脫臼</t>
+    </r>
+  </si>
+  <si>
+    <t>Reimburses 70% of the costs for prescribed FIP treatment medication GS-441524, and supports treatment courses of up to 84 days.
+賠償治療FIP處方藥物GS-441524的7成費用，並支援最長84日療程。</t>
+  </si>
+  <si>
+    <t>one degree</t>
+  </si>
+  <si>
+    <t>ProductID</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="169" formatCode="00000"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -105,6 +208,26 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF667278"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF667278"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -124,10 +247,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -138,14 +262,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -544,15 +692,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A8A0F1C-AF62-9F43-9025-41DFC27676EC}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.6640625" customWidth="1"/>
-    <col min="2" max="2" width="23.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="23.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="29.83203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="66.1640625" customWidth="1"/>
+    <col min="18" max="18" width="45" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -560,48 +719,525 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="P1" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q1" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="S1" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="14">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="5">
+      <c r="E2" s="6">
         <v>30000</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C3" s="3" t="s">
+      <c r="F2" s="6">
+        <v>1</v>
+      </c>
+      <c r="G2" s="6">
+        <v>1</v>
+      </c>
+      <c r="H2" s="6">
+        <v>1</v>
+      </c>
+      <c r="I2" s="6">
+        <v>1</v>
+      </c>
+      <c r="J2" s="6">
+        <v>1</v>
+      </c>
+      <c r="K2" s="6">
+        <v>1</v>
+      </c>
+      <c r="L2" s="6">
+        <v>0</v>
+      </c>
+      <c r="M2" s="6">
+        <v>0</v>
+      </c>
+      <c r="N2" s="6">
+        <v>0</v>
+      </c>
+      <c r="O2" s="6">
+        <v>10000</v>
+      </c>
+      <c r="P2" s="6">
+        <v>10000</v>
+      </c>
+      <c r="Q2" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="R2" s="4">
+        <v>25000</v>
+      </c>
+      <c r="S2" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="3"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="14">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="6">
+        <v>30000</v>
+      </c>
+      <c r="F3" s="6">
+        <v>1</v>
+      </c>
+      <c r="G3" s="6">
+        <v>1</v>
+      </c>
+      <c r="H3" s="6">
+        <v>1</v>
+      </c>
+      <c r="I3" s="6">
+        <v>1</v>
+      </c>
+      <c r="J3" s="6">
+        <v>1</v>
+      </c>
+      <c r="K3" s="6">
+        <v>1</v>
+      </c>
+      <c r="L3" s="6">
+        <v>0</v>
+      </c>
+      <c r="M3" s="6">
+        <v>0</v>
+      </c>
+      <c r="N3" s="6">
+        <v>0</v>
+      </c>
+      <c r="O3" s="6">
+        <v>10000</v>
+      </c>
+      <c r="P3" s="6">
+        <v>10000</v>
+      </c>
+      <c r="Q3" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="R3" s="4">
+        <v>25000</v>
+      </c>
+      <c r="S3" s="11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C4" s="14">
+        <v>3</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="5">
+      <c r="E4" s="6">
         <v>50000</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C4" s="3" t="s">
+      <c r="F4" s="6">
+        <v>1</v>
+      </c>
+      <c r="G4" s="6">
+        <v>1</v>
+      </c>
+      <c r="H4" s="6">
+        <v>1</v>
+      </c>
+      <c r="I4" s="6">
+        <v>1</v>
+      </c>
+      <c r="J4" s="6">
+        <v>1</v>
+      </c>
+      <c r="K4" s="6">
+        <v>1</v>
+      </c>
+      <c r="L4" s="6">
+        <v>1</v>
+      </c>
+      <c r="M4" s="6">
+        <v>1</v>
+      </c>
+      <c r="N4" s="6">
+        <v>0</v>
+      </c>
+      <c r="O4" s="6">
+        <v>10000</v>
+      </c>
+      <c r="P4" s="6">
+        <v>10000</v>
+      </c>
+      <c r="Q4" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="R4" s="4">
+        <v>25000</v>
+      </c>
+      <c r="S4" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C5" s="14">
+        <v>4</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="6">
+        <v>50000</v>
+      </c>
+      <c r="F5" s="6">
+        <v>1</v>
+      </c>
+      <c r="G5" s="6">
+        <v>1</v>
+      </c>
+      <c r="H5" s="6">
+        <v>1</v>
+      </c>
+      <c r="I5" s="6">
+        <v>1</v>
+      </c>
+      <c r="J5" s="6">
+        <v>1</v>
+      </c>
+      <c r="K5" s="6">
+        <v>1</v>
+      </c>
+      <c r="L5" s="6">
+        <v>1</v>
+      </c>
+      <c r="M5" s="6">
+        <v>1</v>
+      </c>
+      <c r="N5" s="6">
+        <v>0</v>
+      </c>
+      <c r="O5" s="6">
+        <v>10000</v>
+      </c>
+      <c r="P5" s="6">
+        <v>10000</v>
+      </c>
+      <c r="Q5" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="R5" s="4">
+        <v>25000</v>
+      </c>
+      <c r="S5" s="11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C6" s="14">
+        <v>5</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="5">
+      <c r="E6" s="6">
         <v>100000</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C5" s="3" t="s">
+      <c r="F6" s="6">
+        <v>1</v>
+      </c>
+      <c r="G6" s="6">
+        <v>1</v>
+      </c>
+      <c r="H6" s="6">
+        <v>1</v>
+      </c>
+      <c r="I6" s="6">
+        <v>1</v>
+      </c>
+      <c r="J6" s="6">
+        <v>1</v>
+      </c>
+      <c r="K6" s="6">
+        <v>1</v>
+      </c>
+      <c r="L6" s="6">
+        <v>1</v>
+      </c>
+      <c r="M6" s="6">
+        <v>1</v>
+      </c>
+      <c r="N6" s="6">
+        <v>0</v>
+      </c>
+      <c r="O6" s="6">
+        <v>10000</v>
+      </c>
+      <c r="P6" s="6">
+        <v>10000</v>
+      </c>
+      <c r="Q6" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="R6" s="4">
+        <v>25000</v>
+      </c>
+      <c r="S6" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C7" s="14">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="6">
+        <v>100000</v>
+      </c>
+      <c r="F7" s="6">
+        <v>1</v>
+      </c>
+      <c r="G7" s="6">
+        <v>1</v>
+      </c>
+      <c r="H7" s="6">
+        <v>1</v>
+      </c>
+      <c r="I7" s="6">
+        <v>1</v>
+      </c>
+      <c r="J7" s="6">
+        <v>1</v>
+      </c>
+      <c r="K7" s="6">
+        <v>1</v>
+      </c>
+      <c r="L7" s="6">
+        <v>1</v>
+      </c>
+      <c r="M7" s="6">
+        <v>1</v>
+      </c>
+      <c r="N7" s="6">
+        <v>0</v>
+      </c>
+      <c r="O7" s="6">
+        <v>10000</v>
+      </c>
+      <c r="P7" s="6">
+        <v>10000</v>
+      </c>
+      <c r="Q7" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="R7" s="4">
+        <v>25000</v>
+      </c>
+      <c r="S7" s="11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C8" s="14">
         <v>7</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D8" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="6">
         <v>100000</v>
+      </c>
+      <c r="F8" s="6">
+        <v>1</v>
+      </c>
+      <c r="G8" s="6">
+        <v>1</v>
+      </c>
+      <c r="H8" s="6">
+        <v>1</v>
+      </c>
+      <c r="I8" s="6">
+        <v>1</v>
+      </c>
+      <c r="J8" s="6">
+        <v>1</v>
+      </c>
+      <c r="K8" s="6">
+        <v>1</v>
+      </c>
+      <c r="L8" s="6">
+        <v>1</v>
+      </c>
+      <c r="M8" s="6">
+        <v>1</v>
+      </c>
+      <c r="N8" s="6">
+        <v>1</v>
+      </c>
+      <c r="O8" s="6">
+        <v>10000</v>
+      </c>
+      <c r="P8" s="6">
+        <v>10000</v>
+      </c>
+      <c r="Q8" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="R8" s="4">
+        <v>25000</v>
+      </c>
+      <c r="S8" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C9" s="14">
+        <v>8</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="6">
+        <v>100000</v>
+      </c>
+      <c r="F9" s="6">
+        <v>1</v>
+      </c>
+      <c r="G9" s="6">
+        <v>1</v>
+      </c>
+      <c r="H9" s="6">
+        <v>1</v>
+      </c>
+      <c r="I9" s="6">
+        <v>1</v>
+      </c>
+      <c r="J9" s="6">
+        <v>1</v>
+      </c>
+      <c r="K9" s="6">
+        <v>1</v>
+      </c>
+      <c r="L9" s="6">
+        <v>1</v>
+      </c>
+      <c r="M9" s="6">
+        <v>1</v>
+      </c>
+      <c r="N9" s="6">
+        <v>1</v>
+      </c>
+      <c r="O9" s="6">
+        <v>10000</v>
+      </c>
+      <c r="P9" s="6">
+        <v>10000</v>
+      </c>
+      <c r="Q9" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="R9" s="4">
+        <v>25000</v>
+      </c>
+      <c r="S9" s="11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="D10" s="3"/>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="D11" s="3"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="P1" location="Glossary!A2" display="Glossary!A2" xr:uid="{37D8FE63-66C4-1C4F-8BA6-CFA90BC99574}"/>
+    <hyperlink ref="R1" location="Glossary!A3" display="Feline Infectious Peritonitis (FIP) Additional Coverage (Cat Only)" xr:uid="{2E72EE70-3AC9-BA46-8A46-99AD4069458C}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{325BD6CE-A468-6B44-9917-405F597C215C}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="41" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="133" x14ac:dyDescent="0.2">
+      <c r="A3" s="13" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>